<commit_message>
ci: optimize workflow for live GitHub Pages deployment and 1200 multi-domain test execution
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Summary_Report.xlsx
+++ b/automation/reports/Excel/Summary_Report.xlsx
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.4</v>
+        <v>0.405</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.335</v>
+        <v>0.342</v>
       </c>
     </row>
     <row r="4">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.241</v>
+        <v>0.243</v>
       </c>
     </row>
     <row r="5">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.2</v>
+        <v>0.196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(cicd): complete Phase 7 CI/CD deployment pipeline, Selenium/Appium/Vulnerability/Load 1200 E2E test suite, and artifact reporting
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Summary_Report.xlsx
+++ b/automation/reports/Excel/Summary_Report.xlsx
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.342</v>
+        <v>0.322</v>
       </c>
     </row>
     <row r="4">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.243</v>
+        <v>0.256</v>
       </c>
     </row>
     <row r="5">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.196</v>
+        <v>0.194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>